<commit_message>
Fill Jul–Sep 2026 actuals from bank statement
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Svhf5NHex7noeB6wTZEiZM
</commit_message>
<xml_diff>
--- a/finance/finance_plan.xlsx
+++ b/finance/finance_plan.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="141">
   <si>
     <t xml:space="preserve">Личный финансовый план — как пользоваться</t>
   </si>
@@ -69,6 +69,9 @@
     <t xml:space="preserve">Бюджет: доходы и расходы по месяцам (факт)</t>
   </si>
   <si>
+    <t xml:space="preserve">Июль–сентябрь 2026: факт из выписки Kaspi Gold. «План/мес» = среднее за эти 3 месяца.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Категория</t>
   </si>
   <si>
@@ -132,7 +135,7 @@
     <t xml:space="preserve">Подработки (нерегулярно, в план не закладываем)</t>
   </si>
   <si>
-    <t xml:space="preserve">Прочие доходы</t>
+    <t xml:space="preserve">Прочие поступления (возвраты от друзей и т.п.)</t>
   </si>
   <si>
     <t xml:space="preserve">Итого: доходы</t>
@@ -150,7 +153,7 @@
     <t xml:space="preserve">Продукты</t>
   </si>
   <si>
-    <t xml:space="preserve">Транспорт</t>
+    <t xml:space="preserve">Транспорт (такси, автобус, бензин)</t>
   </si>
   <si>
     <t xml:space="preserve">Связь и интернет</t>
@@ -165,7 +168,7 @@
     <t xml:space="preserve">Страховки</t>
   </si>
   <si>
-    <t xml:space="preserve">Дети / образование</t>
+    <t xml:space="preserve">IT-сервисы и реклама (работа)</t>
   </si>
   <si>
     <t xml:space="preserve">Итого: обязательные расходы</t>
@@ -174,25 +177,25 @@
     <t xml:space="preserve">Желания</t>
   </si>
   <si>
-    <t xml:space="preserve">Кафе и доставка</t>
+    <t xml:space="preserve">Кафе, рестораны, кофе, доставка</t>
   </si>
   <si>
     <t xml:space="preserve">Желание</t>
   </si>
   <si>
-    <t xml:space="preserve">Развлечения, подписки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Одежда</t>
+    <t xml:space="preserve">Спорт и развлечения</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Одежда, красота, покупки</t>
   </si>
   <si>
     <t xml:space="preserve">Путешествия</t>
   </si>
   <si>
-    <t xml:space="preserve">Подарки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Прочее</t>
+    <t xml:space="preserve">Цветы и подарки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Переводы людям (уточнить), наличные, прочее</t>
   </si>
   <si>
     <t xml:space="preserve">Итого: желания</t>
@@ -1077,7 +1080,9 @@
       <c r="Q1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5"/>
+      <c r="A2" s="5" t="s">
+        <v>14</v>
+      </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -1097,60 +1102,60 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -1171,10 +1176,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5" s="9" t="n">
         <v>1800000</v>
@@ -1185,27 +1190,33 @@
       <c r="G5" s="9"/>
       <c r="H5" s="9"/>
       <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
+      <c r="J5" s="9" t="n">
+        <v>870000</v>
+      </c>
+      <c r="K5" s="9" t="n">
+        <v>1601798</v>
+      </c>
+      <c r="L5" s="9" t="n">
+        <v>1020000</v>
+      </c>
       <c r="M5" s="9"/>
       <c r="N5" s="9"/>
       <c r="O5" s="9"/>
       <c r="P5" s="10" t="n">
         <f aca="false">SUM(D5:O5)</f>
-        <v>0</v>
+        <v>3491798</v>
       </c>
       <c r="Q5" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D5:O5,"&lt;&gt;"),0)</f>
-        <v>0</v>
+        <v>1163932.66666667</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>34</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
@@ -1231,10 +1242,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
@@ -1243,24 +1254,30 @@
       <c r="G7" s="9"/>
       <c r="H7" s="9"/>
       <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
+      <c r="J7" s="9" t="n">
+        <v>119260</v>
+      </c>
+      <c r="K7" s="9" t="n">
+        <v>417729</v>
+      </c>
+      <c r="L7" s="9" t="n">
+        <v>451524</v>
+      </c>
       <c r="M7" s="9"/>
       <c r="N7" s="9"/>
       <c r="O7" s="9"/>
       <c r="P7" s="10" t="n">
         <f aca="false">SUM(D7:O7)</f>
-        <v>0</v>
+        <v>988513</v>
       </c>
       <c r="Q7" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D7:O7,"&lt;&gt;"),0)</f>
-        <v>0</v>
+        <v>329504.333333333</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="12" t="n">
@@ -1293,15 +1310,15 @@
       </c>
       <c r="J8" s="12" t="n">
         <f aca="false">SUM(J5:J7)</f>
-        <v>0</v>
+        <v>989260</v>
       </c>
       <c r="K8" s="12" t="n">
         <f aca="false">SUM(K5:K7)</f>
-        <v>0</v>
+        <v>2019527</v>
       </c>
       <c r="L8" s="12" t="n">
         <f aca="false">SUM(L5:L7)</f>
-        <v>0</v>
+        <v>1471524</v>
       </c>
       <c r="M8" s="12" t="n">
         <f aca="false">SUM(M5:M7)</f>
@@ -1317,11 +1334,11 @@
       </c>
       <c r="P8" s="12" t="n">
         <f aca="false">SUM(P5:P7)</f>
-        <v>0</v>
+        <v>4480311</v>
       </c>
       <c r="Q8" s="12" t="n">
         <f aca="false">SUM(Q5:Q7)</f>
-        <v>0</v>
+        <v>1493437</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1345,7 +1362,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -1366,10 +1383,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
@@ -1395,97 +1412,119 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" s="9"/>
+      <c r="C12" s="9" t="n">
+        <v>304000</v>
+      </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
       <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
+      <c r="J12" s="9" t="n">
+        <v>332451</v>
+      </c>
+      <c r="K12" s="9" t="n">
+        <v>312774</v>
+      </c>
+      <c r="L12" s="9" t="n">
+        <v>266749</v>
+      </c>
       <c r="M12" s="9"/>
       <c r="N12" s="9"/>
       <c r="O12" s="9"/>
       <c r="P12" s="10" t="n">
         <f aca="false">SUM(D12:O12)</f>
-        <v>0</v>
+        <v>911974</v>
       </c>
       <c r="Q12" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D12:O12,"&lt;&gt;"),0)</f>
-        <v>0</v>
+        <v>303991.333333333</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" s="9"/>
+        <v>40</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>171000</v>
+      </c>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9"/>
       <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
+      <c r="J13" s="9" t="n">
+        <v>147665</v>
+      </c>
+      <c r="K13" s="9" t="n">
+        <v>113376</v>
+      </c>
+      <c r="L13" s="9" t="n">
+        <v>251503</v>
+      </c>
       <c r="M13" s="9"/>
       <c r="N13" s="9"/>
       <c r="O13" s="9"/>
       <c r="P13" s="10" t="n">
         <f aca="false">SUM(D13:O13)</f>
-        <v>0</v>
+        <v>512544</v>
       </c>
       <c r="Q13" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D13:O13,"&lt;&gt;"),0)</f>
-        <v>0</v>
+        <v>170848</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C14" s="9"/>
+        <v>40</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>6000</v>
+      </c>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
       <c r="F14" s="9"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
       <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
+      <c r="J14" s="9" t="n">
+        <v>12960</v>
+      </c>
       <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
+      <c r="L14" s="9" t="n">
+        <v>4499</v>
+      </c>
       <c r="M14" s="9"/>
       <c r="N14" s="9"/>
       <c r="O14" s="9"/>
       <c r="P14" s="10" t="n">
         <f aca="false">SUM(D14:O14)</f>
-        <v>0</v>
+        <v>17459</v>
       </c>
       <c r="Q14" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D14:O14,"&lt;&gt;"),0)</f>
-        <v>0</v>
+        <v>8729.5</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
@@ -1511,10 +1550,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
@@ -1540,10 +1579,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
@@ -1569,41 +1608,49 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C18" s="9"/>
+        <v>40</v>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>85000</v>
+      </c>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
       <c r="G18" s="9"/>
       <c r="H18" s="9"/>
       <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
-      <c r="K18" s="9"/>
-      <c r="L18" s="9"/>
+      <c r="J18" s="9" t="n">
+        <v>74890</v>
+      </c>
+      <c r="K18" s="9" t="n">
+        <v>108492</v>
+      </c>
+      <c r="L18" s="9" t="n">
+        <v>73060</v>
+      </c>
       <c r="M18" s="9"/>
       <c r="N18" s="9"/>
       <c r="O18" s="9"/>
       <c r="P18" s="10" t="n">
         <f aca="false">SUM(D18:O18)</f>
-        <v>0</v>
+        <v>256442</v>
       </c>
       <c r="Q18" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D18:O18,"&lt;&gt;"),0)</f>
-        <v>0</v>
+        <v>85480.6666666667</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="12" t="n">
         <f aca="false">SUM(C11:C18)</f>
-        <v>0</v>
+        <v>566000</v>
       </c>
       <c r="D19" s="12" t="n">
         <f aca="false">SUM(D11:D18)</f>
@@ -1631,15 +1678,15 @@
       </c>
       <c r="J19" s="12" t="n">
         <f aca="false">SUM(J11:J18)</f>
-        <v>0</v>
+        <v>567966</v>
       </c>
       <c r="K19" s="12" t="n">
         <f aca="false">SUM(K11:K18)</f>
-        <v>0</v>
+        <v>534642</v>
       </c>
       <c r="L19" s="12" t="n">
         <f aca="false">SUM(L11:L18)</f>
-        <v>0</v>
+        <v>595811</v>
       </c>
       <c r="M19" s="12" t="n">
         <f aca="false">SUM(M11:M18)</f>
@@ -1655,11 +1702,11 @@
       </c>
       <c r="P19" s="12" t="n">
         <f aca="false">SUM(P11:P18)</f>
-        <v>0</v>
+        <v>1698419</v>
       </c>
       <c r="Q19" s="12" t="n">
         <f aca="false">SUM(Q11:Q18)</f>
-        <v>0</v>
+        <v>569049.5</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1683,7 +1730,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -1704,97 +1751,121 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C22" s="9"/>
+        <v>51</v>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>284000</v>
+      </c>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
       <c r="G22" s="9"/>
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
-      <c r="K22" s="9"/>
-      <c r="L22" s="9"/>
+      <c r="J22" s="9" t="n">
+        <v>270414</v>
+      </c>
+      <c r="K22" s="9" t="n">
+        <v>258681</v>
+      </c>
+      <c r="L22" s="9" t="n">
+        <v>323226</v>
+      </c>
       <c r="M22" s="9"/>
       <c r="N22" s="9"/>
       <c r="O22" s="9"/>
       <c r="P22" s="10" t="n">
         <f aca="false">SUM(D22:O22)</f>
-        <v>0</v>
+        <v>852321</v>
       </c>
       <c r="Q22" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D22:O22,"&lt;&gt;"),0)</f>
-        <v>0</v>
+        <v>284107</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B23" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C23" s="9"/>
+      <c r="C23" s="9" t="n">
+        <v>90000</v>
+      </c>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
       <c r="F23" s="9"/>
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
       <c r="I23" s="9"/>
-      <c r="J23" s="9"/>
-      <c r="K23" s="9"/>
-      <c r="L23" s="9"/>
+      <c r="J23" s="9" t="n">
+        <v>62754</v>
+      </c>
+      <c r="K23" s="9" t="n">
+        <v>193281</v>
+      </c>
+      <c r="L23" s="9" t="n">
+        <v>14530</v>
+      </c>
       <c r="M23" s="9"/>
       <c r="N23" s="9"/>
       <c r="O23" s="9"/>
       <c r="P23" s="10" t="n">
         <f aca="false">SUM(D23:O23)</f>
-        <v>0</v>
+        <v>270565</v>
       </c>
       <c r="Q23" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D23:O23,"&lt;&gt;"),0)</f>
-        <v>0</v>
+        <v>90188.3333333333</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C24" s="9"/>
+        <v>51</v>
+      </c>
+      <c r="C24" s="9" t="n">
+        <v>50000</v>
+      </c>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
       <c r="G24" s="9"/>
       <c r="H24" s="9"/>
       <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
-      <c r="K24" s="9"/>
-      <c r="L24" s="9"/>
+      <c r="J24" s="9" t="n">
+        <v>105949</v>
+      </c>
+      <c r="K24" s="9" t="n">
+        <v>27921</v>
+      </c>
+      <c r="L24" s="9" t="n">
+        <v>17482</v>
+      </c>
       <c r="M24" s="9"/>
       <c r="N24" s="9"/>
       <c r="O24" s="9"/>
       <c r="P24" s="10" t="n">
         <f aca="false">SUM(D24:O24)</f>
-        <v>0</v>
+        <v>151352</v>
       </c>
       <c r="Q24" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D24:O24,"&lt;&gt;"),0)</f>
-        <v>0</v>
+        <v>50450.6666666667</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
@@ -1820,70 +1891,86 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C26" s="9"/>
+        <v>51</v>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>14000</v>
+      </c>
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
       <c r="H26" s="9"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="9"/>
-      <c r="K26" s="9"/>
-      <c r="L26" s="9"/>
+      <c r="J26" s="9" t="n">
+        <v>37000</v>
+      </c>
+      <c r="K26" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="L26" s="9" t="n">
+        <v>2000</v>
+      </c>
       <c r="M26" s="9"/>
       <c r="N26" s="9"/>
       <c r="O26" s="9"/>
       <c r="P26" s="10" t="n">
         <f aca="false">SUM(D26:O26)</f>
-        <v>0</v>
+        <v>40500</v>
       </c>
       <c r="Q26" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D26:O26,"&lt;&gt;"),0)</f>
-        <v>0</v>
+        <v>13500</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C27" s="9"/>
+        <v>51</v>
+      </c>
+      <c r="C27" s="9" t="n">
+        <v>656000</v>
+      </c>
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
       <c r="G27" s="9"/>
       <c r="H27" s="9"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
-      <c r="K27" s="9"/>
-      <c r="L27" s="9"/>
+      <c r="J27" s="9" t="n">
+        <v>487961</v>
+      </c>
+      <c r="K27" s="9" t="n">
+        <v>976845</v>
+      </c>
+      <c r="L27" s="9" t="n">
+        <v>504322</v>
+      </c>
       <c r="M27" s="9"/>
       <c r="N27" s="9"/>
       <c r="O27" s="9"/>
       <c r="P27" s="10" t="n">
         <f aca="false">SUM(D27:O27)</f>
-        <v>0</v>
+        <v>1969128</v>
       </c>
       <c r="Q27" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D27:O27,"&lt;&gt;"),0)</f>
-        <v>0</v>
+        <v>656376</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="12" t="n">
         <f aca="false">SUM(C22:C27)</f>
-        <v>0</v>
+        <v>1094000</v>
       </c>
       <c r="D28" s="12" t="n">
         <f aca="false">SUM(D22:D27)</f>
@@ -1911,15 +1998,15 @@
       </c>
       <c r="J28" s="12" t="n">
         <f aca="false">SUM(J22:J27)</f>
-        <v>0</v>
+        <v>964078</v>
       </c>
       <c r="K28" s="12" t="n">
         <f aca="false">SUM(K22:K27)</f>
-        <v>0</v>
+        <v>1458228</v>
       </c>
       <c r="L28" s="12" t="n">
         <f aca="false">SUM(L22:L27)</f>
-        <v>0</v>
+        <v>861560</v>
       </c>
       <c r="M28" s="12" t="n">
         <f aca="false">SUM(M22:M27)</f>
@@ -1935,11 +2022,11 @@
       </c>
       <c r="P28" s="12" t="n">
         <f aca="false">SUM(P22:P27)</f>
-        <v>0</v>
+        <v>3283866</v>
       </c>
       <c r="Q28" s="12" t="n">
         <f aca="false">SUM(Q22:Q27)</f>
-        <v>0</v>
+        <v>1094622</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1963,7 +2050,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="8"/>
@@ -1984,10 +2071,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C31" s="9"/>
       <c r="D31" s="9"/>
@@ -2013,10 +2100,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B32" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>59</v>
       </c>
       <c r="C32" s="9"/>
       <c r="D32" s="9"/>
@@ -2042,10 +2129,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
@@ -2071,7 +2158,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="12" t="n">
@@ -2156,7 +2243,7 @@
     </row>
     <row r="36" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B36" s="5"/>
       <c r="C36" s="5"/>
@@ -2177,12 +2264,12 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B37" s="5"/>
       <c r="C37" s="10" t="n">
         <f aca="false">C8-C19-C28-C34</f>
-        <v>1800000</v>
+        <v>140000</v>
       </c>
       <c r="D37" s="10" t="n">
         <f aca="false">D8-D19-D28-D34</f>
@@ -2210,15 +2297,15 @@
       </c>
       <c r="J37" s="10" t="n">
         <f aca="false">J8-J19-J28-J34</f>
-        <v>0</v>
+        <v>-542784</v>
       </c>
       <c r="K37" s="10" t="n">
         <f aca="false">K8-K19-K28-K34</f>
-        <v>0</v>
+        <v>26657</v>
       </c>
       <c r="L37" s="10" t="n">
         <f aca="false">L8-L19-L28-L34</f>
-        <v>0</v>
+        <v>14153</v>
       </c>
       <c r="M37" s="10" t="n">
         <f aca="false">M8-M19-M28-M34</f>
@@ -2234,21 +2321,21 @@
       </c>
       <c r="P37" s="10" t="n">
         <f aca="false">P8-P19-P28-P34</f>
-        <v>0</v>
+        <v>-501974</v>
       </c>
       <c r="Q37" s="10" t="n">
         <f aca="false">Q8-Q19-Q28-Q34</f>
-        <v>0</v>
+        <v>-170234.5</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B38" s="5"/>
       <c r="C38" s="13" t="n">
         <f aca="false">IFERROR(C19/C8,0)</f>
-        <v>0</v>
+        <v>0.314444444444444</v>
       </c>
       <c r="D38" s="13" t="n">
         <f aca="false">IFERROR(D19/D8,0)</f>
@@ -2276,15 +2363,15 @@
       </c>
       <c r="J38" s="13" t="n">
         <f aca="false">IFERROR(J19/J8,0)</f>
-        <v>0</v>
+        <v>0.574132179609001</v>
       </c>
       <c r="K38" s="13" t="n">
         <f aca="false">IFERROR(K19/K8,0)</f>
-        <v>0</v>
+        <v>0.264736247646107</v>
       </c>
       <c r="L38" s="13" t="n">
         <f aca="false">IFERROR(L19/L8,0)</f>
-        <v>0</v>
+        <v>0.404893837953034</v>
       </c>
       <c r="M38" s="13" t="n">
         <f aca="false">IFERROR(M19/M8,0)</f>
@@ -2300,21 +2387,21 @@
       </c>
       <c r="P38" s="13" t="n">
         <f aca="false">IFERROR(P19/P8,0)</f>
-        <v>0</v>
+        <v>0.37908506797854</v>
       </c>
       <c r="Q38" s="13" t="n">
         <f aca="false">IFERROR(Q19/Q8,0)</f>
-        <v>0</v>
+        <v>0.381033481827489</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="13" t="n">
         <f aca="false">IFERROR(C28/C8,0)</f>
-        <v>0</v>
+        <v>0.607777777777778</v>
       </c>
       <c r="D39" s="13" t="n">
         <f aca="false">IFERROR(D28/D8,0)</f>
@@ -2342,15 +2429,15 @@
       </c>
       <c r="J39" s="13" t="n">
         <f aca="false">IFERROR(J28/J8,0)</f>
-        <v>0</v>
+        <v>0.974544609101753</v>
       </c>
       <c r="K39" s="13" t="n">
         <f aca="false">IFERROR(K28/K8,0)</f>
-        <v>0</v>
+        <v>0.722064126897041</v>
       </c>
       <c r="L39" s="13" t="n">
         <f aca="false">IFERROR(L28/L8,0)</f>
-        <v>0</v>
+        <v>0.585488242121773</v>
       </c>
       <c r="M39" s="13" t="n">
         <f aca="false">IFERROR(M28/M8,0)</f>
@@ -2366,16 +2453,16 @@
       </c>
       <c r="P39" s="13" t="n">
         <f aca="false">IFERROR(P28/P8,0)</f>
-        <v>0</v>
+        <v>0.732954922102506</v>
       </c>
       <c r="Q39" s="13" t="n">
         <f aca="false">IFERROR(Q28/Q8,0)</f>
-        <v>0</v>
+        <v>0.732954922102506</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B40" s="5"/>
       <c r="C40" s="13" t="n">
@@ -2460,7 +2547,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B42" s="5"/>
       <c r="C42" s="5"/>
@@ -2481,7 +2568,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B43" s="5"/>
       <c r="C43" s="14" t="n">
@@ -2504,7 +2591,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B44" s="5"/>
       <c r="C44" s="14" t="n">
@@ -2527,7 +2614,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B45" s="5"/>
       <c r="C45" s="14" t="n">
@@ -2550,7 +2637,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B46" s="5"/>
       <c r="C46" s="5"/>
@@ -2596,7 +2683,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -2604,7 +2691,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="16"/>
@@ -2618,100 +2705,100 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C6" s="9"/>
       <c r="D6" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C8" s="9"/>
       <c r="D8" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C9" s="9"/>
       <c r="D9" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C10" s="9"/>
       <c r="D10" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C11" s="9"/>
       <c r="D11" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2734,7 +2821,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="12" t="n">
@@ -2745,7 +2832,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16" s="10" t="n">
@@ -2762,62 +2849,62 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B20" s="5" t="s">
         <v>96</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>95</v>
       </c>
       <c r="C20" s="9"/>
       <c r="D20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C21" s="9"/>
       <c r="D21" s="5"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C22" s="9"/>
       <c r="D22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C23" s="9"/>
       <c r="D23" s="5"/>
@@ -2836,7 +2923,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B26" s="5"/>
       <c r="C26" s="12" t="n">
@@ -2853,7 +2940,7 @@
     </row>
     <row r="28" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="17" t="n">
@@ -2893,7 +2980,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B1" s="5"/>
     </row>
@@ -2903,31 +2990,31 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B3" s="18" t="n">
         <f aca="false">Бюджет!Q19</f>
-        <v>0</v>
+        <v>569049.5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B5" s="19" t="n">
         <f aca="false">IF(B4&gt;0,B4,B3)</f>
-        <v>0</v>
+        <v>569049.5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B6" s="20" t="n">
         <v>6</v>
@@ -2935,16 +3022,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B7" s="12" t="n">
         <f aca="false">B5*B6</f>
-        <v>0</v>
+        <v>3414297</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B8" s="18" t="n">
         <f aca="false">Капитал!C16</f>
@@ -2953,16 +3040,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B9" s="12" t="n">
         <f aca="false">MAX(0,B7-B8)</f>
-        <v>0</v>
+        <v>3414297</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B10" s="21" t="n">
         <f aca="false">IFERROR(MIN(1,B8/B7),0)</f>
@@ -2971,17 +3058,17 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="B12" s="22" t="n">
+        <v>113</v>
+      </c>
+      <c r="B12" s="22" t="str">
         <f aca="false">IF(B9=0,0,IFERROR(ROUNDUP(B9/B11,0),"укажите взнос"))</f>
-        <v>0</v>
+        <v>укажите взнос</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2990,7 +3077,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B14" s="5"/>
     </row>
@@ -3025,7 +3112,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -3038,7 +3125,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B2" s="23" t="n">
         <f aca="true">TODAY()</f>
@@ -3065,36 +3152,36 @@
     </row>
     <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>2</v>
@@ -3345,7 +3432,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -3361,7 +3448,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -3401,7 +3488,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -3413,7 +3500,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -3435,33 +3522,33 @@
     </row>
     <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B5" s="9" t="n">
         <v>600000</v>
@@ -3633,7 +3720,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">SUM(B5:B12)</f>
@@ -3660,7 +3747,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>

</xml_diff>

<commit_message>
Reclassify transfers, add cash rent and utilities to Jul–Sep budget
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Svhf5NHex7noeB6wTZEiZM
</commit_message>
<xml_diff>
--- a/finance/finance_plan.xlsx
+++ b/finance/finance_plan.xlsx
@@ -69,7 +69,7 @@
     <t xml:space="preserve">Бюджет: доходы и расходы по месяцам (факт)</t>
   </si>
   <si>
-    <t xml:space="preserve">Июль–сентябрь 2026: факт из выписки Kaspi Gold. «План/мес» = среднее за эти 3 месяца.</t>
+    <t xml:space="preserve">Июль–сентябрь 2026: факт по выписке Kaspi + аренда и коммуналка наличными. Транзит через Дидара (403 тыс.) исключён. «План/мес» = среднее за 3 мес., без зарплаты Александре (прекращено) и без возвратов от друзей.</t>
   </si>
   <si>
     <t xml:space="preserve">Категория</t>
@@ -135,7 +135,7 @@
     <t xml:space="preserve">Подработки (нерегулярно, в план не закладываем)</t>
   </si>
   <si>
-    <t xml:space="preserve">Прочие поступления (возвраты от друзей и т.п.)</t>
+    <t xml:space="preserve">Возвраты от друзей и прочие поступления</t>
   </si>
   <si>
     <t xml:space="preserve">Итого: доходы</t>
@@ -144,7 +144,7 @@
     <t xml:space="preserve">Обязательные расходы</t>
   </si>
   <si>
-    <t xml:space="preserve">Жильё (аренда/ипотека, коммуналка)</t>
+    <t xml:space="preserve">Жильё: аренда 450 тыс. + коммуналка ~27,5 тыс. (наличными)</t>
   </si>
   <si>
     <t xml:space="preserve">Обязательное</t>
@@ -165,7 +165,7 @@
     <t xml:space="preserve">Платежи по долгам (минимальные)</t>
   </si>
   <si>
-    <t xml:space="preserve">Страховки</t>
+    <t xml:space="preserve">Налоги</t>
   </si>
   <si>
     <t xml:space="preserve">IT-сервисы и реклама (работа)</t>
@@ -189,13 +189,13 @@
     <t xml:space="preserve">Одежда, красота, покупки</t>
   </si>
   <si>
-    <t xml:space="preserve">Путешествия</t>
+    <t xml:space="preserve">Боулинг (тренер, инвентарь, игры)</t>
   </si>
   <si>
     <t xml:space="preserve">Цветы и подарки</t>
   </si>
   <si>
-    <t xml:space="preserve">Переводы людям (уточнить), наличные, прочее</t>
+    <t xml:space="preserve">Прочие переводы, супруге, наличные, прочее</t>
   </si>
   <si>
     <t xml:space="preserve">Итого: желания</t>
@@ -1191,24 +1191,24 @@
       <c r="H5" s="9"/>
       <c r="I5" s="9"/>
       <c r="J5" s="9" t="n">
-        <v>870000</v>
+        <v>1319900</v>
       </c>
       <c r="K5" s="9" t="n">
-        <v>1601798</v>
+        <v>1897398</v>
       </c>
       <c r="L5" s="9" t="n">
-        <v>1020000</v>
+        <v>1303700</v>
       </c>
       <c r="M5" s="9"/>
       <c r="N5" s="9"/>
       <c r="O5" s="9"/>
       <c r="P5" s="10" t="n">
         <f aca="false">SUM(D5:O5)</f>
-        <v>3491798</v>
+        <v>4520998</v>
       </c>
       <c r="Q5" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D5:O5,"&lt;&gt;"),0)</f>
-        <v>1163932.66666667</v>
+        <v>1506999.33333333</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1247,7 +1247,9 @@
       <c r="B7" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="9"/>
+      <c r="C7" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
@@ -1255,24 +1257,24 @@
       <c r="H7" s="9"/>
       <c r="I7" s="9"/>
       <c r="J7" s="9" t="n">
-        <v>119260</v>
+        <v>53260</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>417729</v>
+        <v>297229</v>
       </c>
       <c r="L7" s="9" t="n">
-        <v>451524</v>
+        <v>382594</v>
       </c>
       <c r="M7" s="9"/>
       <c r="N7" s="9"/>
       <c r="O7" s="9"/>
       <c r="P7" s="10" t="n">
         <f aca="false">SUM(D7:O7)</f>
-        <v>988513</v>
+        <v>733083</v>
       </c>
       <c r="Q7" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D7:O7,"&lt;&gt;"),0)</f>
-        <v>329504.333333333</v>
+        <v>244361</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1310,15 +1312,15 @@
       </c>
       <c r="J8" s="12" t="n">
         <f aca="false">SUM(J5:J7)</f>
-        <v>989260</v>
+        <v>1373160</v>
       </c>
       <c r="K8" s="12" t="n">
         <f aca="false">SUM(K5:K7)</f>
-        <v>2019527</v>
+        <v>2194627</v>
       </c>
       <c r="L8" s="12" t="n">
         <f aca="false">SUM(L5:L7)</f>
-        <v>1471524</v>
+        <v>1686294</v>
       </c>
       <c r="M8" s="12" t="n">
         <f aca="false">SUM(M5:M7)</f>
@@ -1334,11 +1336,11 @@
       </c>
       <c r="P8" s="12" t="n">
         <f aca="false">SUM(P5:P7)</f>
-        <v>4480311</v>
+        <v>5254081</v>
       </c>
       <c r="Q8" s="12" t="n">
         <f aca="false">SUM(Q5:Q7)</f>
-        <v>1493437</v>
+        <v>1751360.33333333</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1388,26 +1390,34 @@
       <c r="B11" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C11" s="9"/>
+      <c r="C11" s="9" t="n">
+        <v>478000</v>
+      </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
       <c r="F11" s="9"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
+      <c r="J11" s="9" t="n">
+        <v>477500</v>
+      </c>
+      <c r="K11" s="9" t="n">
+        <v>477500</v>
+      </c>
+      <c r="L11" s="9" t="n">
+        <v>477500</v>
+      </c>
       <c r="M11" s="9"/>
       <c r="N11" s="9"/>
       <c r="O11" s="9"/>
       <c r="P11" s="10" t="n">
         <f aca="false">SUM(D11:O11)</f>
-        <v>0</v>
+        <v>1432500</v>
       </c>
       <c r="Q11" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D11:O11,"&lt;&gt;"),0)</f>
-        <v>0</v>
+        <v>477500</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1418,7 +1428,7 @@
         <v>40</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>304000</v>
+        <v>329000</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
@@ -1427,24 +1437,24 @@
       <c r="H12" s="9"/>
       <c r="I12" s="9"/>
       <c r="J12" s="9" t="n">
-        <v>332451</v>
+        <v>382991</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>312774</v>
+        <v>330674</v>
       </c>
       <c r="L12" s="9" t="n">
-        <v>266749</v>
+        <v>274329</v>
       </c>
       <c r="M12" s="9"/>
       <c r="N12" s="9"/>
       <c r="O12" s="9"/>
       <c r="P12" s="10" t="n">
         <f aca="false">SUM(D12:O12)</f>
-        <v>911974</v>
+        <v>987994</v>
       </c>
       <c r="Q12" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D12:O12,"&lt;&gt;"),0)</f>
-        <v>303991.333333333</v>
+        <v>329331.333333333</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1584,7 +1594,9 @@
       <c r="B17" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="9"/>
+      <c r="C17" s="9" t="n">
+        <v>27000</v>
+      </c>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
@@ -1592,18 +1604,22 @@
       <c r="H17" s="9"/>
       <c r="I17" s="9"/>
       <c r="J17" s="9"/>
-      <c r="K17" s="9"/>
-      <c r="L17" s="9"/>
+      <c r="K17" s="9" t="n">
+        <v>79900</v>
+      </c>
+      <c r="L17" s="9" t="n">
+        <v>1650</v>
+      </c>
       <c r="M17" s="9"/>
       <c r="N17" s="9"/>
       <c r="O17" s="9"/>
       <c r="P17" s="10" t="n">
         <f aca="false">SUM(D17:O17)</f>
-        <v>0</v>
+        <v>81550</v>
       </c>
       <c r="Q17" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D17:O17,"&lt;&gt;"),0)</f>
-        <v>0</v>
+        <v>40775</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1650,7 +1666,7 @@
       <c r="B19" s="5"/>
       <c r="C19" s="12" t="n">
         <f aca="false">SUM(C11:C18)</f>
-        <v>566000</v>
+        <v>1096000</v>
       </c>
       <c r="D19" s="12" t="n">
         <f aca="false">SUM(D11:D18)</f>
@@ -1678,15 +1694,15 @@
       </c>
       <c r="J19" s="12" t="n">
         <f aca="false">SUM(J11:J18)</f>
-        <v>567966</v>
+        <v>1096006</v>
       </c>
       <c r="K19" s="12" t="n">
         <f aca="false">SUM(K11:K18)</f>
-        <v>534642</v>
+        <v>1109942</v>
       </c>
       <c r="L19" s="12" t="n">
         <f aca="false">SUM(L11:L18)</f>
-        <v>595811</v>
+        <v>1082541</v>
       </c>
       <c r="M19" s="12" t="n">
         <f aca="false">SUM(M11:M18)</f>
@@ -1702,11 +1718,11 @@
       </c>
       <c r="P19" s="12" t="n">
         <f aca="false">SUM(P11:P18)</f>
-        <v>1698419</v>
+        <v>3288489</v>
       </c>
       <c r="Q19" s="12" t="n">
         <f aca="false">SUM(Q11:Q18)</f>
-        <v>569049.5</v>
+        <v>1112664.5</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1757,7 +1773,7 @@
         <v>51</v>
       </c>
       <c r="C22" s="9" t="n">
-        <v>284000</v>
+        <v>292000</v>
       </c>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
@@ -1766,24 +1782,24 @@
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
       <c r="J22" s="9" t="n">
-        <v>270414</v>
+        <v>275024</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>258681</v>
+        <v>269661</v>
       </c>
       <c r="L22" s="9" t="n">
-        <v>323226</v>
+        <v>331096</v>
       </c>
       <c r="M22" s="9"/>
       <c r="N22" s="9"/>
       <c r="O22" s="9"/>
       <c r="P22" s="10" t="n">
         <f aca="false">SUM(D22:O22)</f>
-        <v>852321</v>
+        <v>875781</v>
       </c>
       <c r="Q22" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D22:O22,"&lt;&gt;"),0)</f>
-        <v>284107</v>
+        <v>291927</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1794,7 +1810,7 @@
         <v>51</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>90000</v>
+        <v>52000</v>
       </c>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
@@ -1803,10 +1819,10 @@
       <c r="H23" s="9"/>
       <c r="I23" s="9"/>
       <c r="J23" s="9" t="n">
-        <v>62754</v>
+        <v>12664</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>193281</v>
+        <v>128384</v>
       </c>
       <c r="L23" s="9" t="n">
         <v>14530</v>
@@ -1816,11 +1832,11 @@
       <c r="O23" s="9"/>
       <c r="P23" s="10" t="n">
         <f aca="false">SUM(D23:O23)</f>
-        <v>270565</v>
+        <v>155578</v>
       </c>
       <c r="Q23" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D23:O23,"&lt;&gt;"),0)</f>
-        <v>90188.3333333333</v>
+        <v>51859.3333333333</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1867,26 +1883,34 @@
       <c r="B25" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="9"/>
+      <c r="C25" s="9" t="n">
+        <v>150000</v>
+      </c>
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
       <c r="H25" s="9"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
-      <c r="K25" s="9"/>
-      <c r="L25" s="9"/>
+      <c r="J25" s="9" t="n">
+        <v>97090</v>
+      </c>
+      <c r="K25" s="9" t="n">
+        <v>273897</v>
+      </c>
+      <c r="L25" s="9" t="n">
+        <v>80000</v>
+      </c>
       <c r="M25" s="9"/>
       <c r="N25" s="9"/>
       <c r="O25" s="9"/>
       <c r="P25" s="10" t="n">
         <f aca="false">SUM(D25:O25)</f>
-        <v>0</v>
+        <v>450987</v>
       </c>
       <c r="Q25" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D25:O25,"&lt;&gt;"),0)</f>
-        <v>0</v>
+        <v>150329</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1934,7 +1958,7 @@
         <v>51</v>
       </c>
       <c r="C27" s="9" t="n">
-        <v>656000</v>
+        <v>159000</v>
       </c>
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
@@ -1943,24 +1967,24 @@
       <c r="H27" s="9"/>
       <c r="I27" s="9"/>
       <c r="J27" s="9" t="n">
-        <v>487961</v>
+        <v>292211</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>976845</v>
+        <v>356665</v>
       </c>
       <c r="L27" s="9" t="n">
-        <v>504322</v>
+        <v>144492</v>
       </c>
       <c r="M27" s="9"/>
       <c r="N27" s="9"/>
       <c r="O27" s="9"/>
       <c r="P27" s="10" t="n">
         <f aca="false">SUM(D27:O27)</f>
-        <v>1969128</v>
+        <v>793368</v>
       </c>
       <c r="Q27" s="10" t="n">
         <f aca="false">IFERROR(AVERAGEIF(D27:O27,"&lt;&gt;"),0)</f>
-        <v>656376</v>
+        <v>264456</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1970,7 +1994,7 @@
       <c r="B28" s="5"/>
       <c r="C28" s="12" t="n">
         <f aca="false">SUM(C22:C27)</f>
-        <v>1094000</v>
+        <v>717000</v>
       </c>
       <c r="D28" s="12" t="n">
         <f aca="false">SUM(D22:D27)</f>
@@ -1998,15 +2022,15 @@
       </c>
       <c r="J28" s="12" t="n">
         <f aca="false">SUM(J22:J27)</f>
-        <v>964078</v>
+        <v>819938</v>
       </c>
       <c r="K28" s="12" t="n">
         <f aca="false">SUM(K22:K27)</f>
-        <v>1458228</v>
+        <v>1058028</v>
       </c>
       <c r="L28" s="12" t="n">
         <f aca="false">SUM(L22:L27)</f>
-        <v>861560</v>
+        <v>589600</v>
       </c>
       <c r="M28" s="12" t="n">
         <f aca="false">SUM(M22:M27)</f>
@@ -2022,11 +2046,11 @@
       </c>
       <c r="P28" s="12" t="n">
         <f aca="false">SUM(P22:P27)</f>
-        <v>3283866</v>
+        <v>2467566</v>
       </c>
       <c r="Q28" s="12" t="n">
         <f aca="false">SUM(Q22:Q27)</f>
-        <v>1094622</v>
+        <v>822522</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2269,7 +2293,7 @@
       <c r="B37" s="5"/>
       <c r="C37" s="10" t="n">
         <f aca="false">C8-C19-C28-C34</f>
-        <v>140000</v>
+        <v>-13000</v>
       </c>
       <c r="D37" s="10" t="n">
         <f aca="false">D8-D19-D28-D34</f>
@@ -2325,7 +2349,7 @@
       </c>
       <c r="Q37" s="10" t="n">
         <f aca="false">Q8-Q19-Q28-Q34</f>
-        <v>-170234.5</v>
+        <v>-183826.166666667</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2335,7 +2359,7 @@
       <c r="B38" s="5"/>
       <c r="C38" s="13" t="n">
         <f aca="false">IFERROR(C19/C8,0)</f>
-        <v>0.314444444444444</v>
+        <v>0.608888888888889</v>
       </c>
       <c r="D38" s="13" t="n">
         <f aca="false">IFERROR(D19/D8,0)</f>
@@ -2363,15 +2387,15 @@
       </c>
       <c r="J38" s="13" t="n">
         <f aca="false">IFERROR(J19/J8,0)</f>
-        <v>0.574132179609001</v>
+        <v>0.798163360424131</v>
       </c>
       <c r="K38" s="13" t="n">
         <f aca="false">IFERROR(K19/K8,0)</f>
-        <v>0.264736247646107</v>
+        <v>0.50575428079578</v>
       </c>
       <c r="L38" s="13" t="n">
         <f aca="false">IFERROR(L19/L8,0)</f>
-        <v>0.404893837953034</v>
+        <v>0.641964568456034</v>
       </c>
       <c r="M38" s="13" t="n">
         <f aca="false">IFERROR(M19/M8,0)</f>
@@ -2387,11 +2411,11 @@
       </c>
       <c r="P38" s="13" t="n">
         <f aca="false">IFERROR(P19/P8,0)</f>
-        <v>0.37908506797854</v>
+        <v>0.625892330171537</v>
       </c>
       <c r="Q38" s="13" t="n">
         <f aca="false">IFERROR(Q19/Q8,0)</f>
-        <v>0.381033481827489</v>
+        <v>0.635314434627102</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2401,7 +2425,7 @@
       <c r="B39" s="5"/>
       <c r="C39" s="13" t="n">
         <f aca="false">IFERROR(C28/C8,0)</f>
-        <v>0.607777777777778</v>
+        <v>0.398333333333333</v>
       </c>
       <c r="D39" s="13" t="n">
         <f aca="false">IFERROR(D28/D8,0)</f>
@@ -2429,15 +2453,15 @@
       </c>
       <c r="J39" s="13" t="n">
         <f aca="false">IFERROR(J28/J8,0)</f>
-        <v>0.974544609101753</v>
+        <v>0.597117597366658</v>
       </c>
       <c r="K39" s="13" t="n">
         <f aca="false">IFERROR(K28/K8,0)</f>
-        <v>0.722064126897041</v>
+        <v>0.482099235997734</v>
       </c>
       <c r="L39" s="13" t="n">
         <f aca="false">IFERROR(L28/L8,0)</f>
-        <v>0.585488242121773</v>
+        <v>0.349642470411447</v>
       </c>
       <c r="M39" s="13" t="n">
         <f aca="false">IFERROR(M28/M8,0)</f>
@@ -2453,11 +2477,11 @@
       </c>
       <c r="P39" s="13" t="n">
         <f aca="false">IFERROR(P28/P8,0)</f>
-        <v>0.732954922102506</v>
+        <v>0.469647498772859</v>
       </c>
       <c r="Q39" s="13" t="n">
         <f aca="false">IFERROR(Q28/Q8,0)</f>
-        <v>0.732954922102506</v>
+        <v>0.469647498772859</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2994,7 +3018,7 @@
       </c>
       <c r="B3" s="18" t="n">
         <f aca="false">Бюджет!Q19</f>
-        <v>569049.5</v>
+        <v>1112664.5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3009,7 +3033,7 @@
       </c>
       <c r="B5" s="19" t="n">
         <f aca="false">IF(B4&gt;0,B4,B3)</f>
-        <v>569049.5</v>
+        <v>1112664.5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3026,7 +3050,7 @@
       </c>
       <c r="B7" s="12" t="n">
         <f aca="false">B5*B6</f>
-        <v>3414297</v>
+        <v>6675987</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3044,7 +3068,7 @@
       </c>
       <c r="B9" s="12" t="n">
         <f aca="false">MAX(0,B7-B8)</f>
-        <v>3414297</v>
+        <v>6675987</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>